<commit_message>
feat(main): ejecución por Excel con timeout, exportación de resultados y .gitignore
</commit_message>
<xml_diff>
--- a/results/resultados_Geometric.xlsx
+++ b/results/resultados_Geometric.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,11 +447,6 @@
           <t>Tiempo de ejecución (s)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -459,31 +454,30 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>| A,B,C,E,F,G,H,I,J || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| H || A,B,C,D,E,F,G,I,J,K,L,M,N,O |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0,02536296844482422</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>1,573875904083252</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -491,31 +485,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>|   A,B,C,D,E,F,H,I   || G |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| H || A,B,C,D,E,F,G,I,J,K,L,M,N,O |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0,00026786327</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0,04569554328918457</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>1,6588985919952393</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -523,31 +516,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>|   B,C,D,E,F,H,I,J   || G |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| B || A,C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o ||  b,c,d,e,f,g,h,i,j,k,l,m,n  |</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0,00026786327</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0,04589223861694336</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>0,911250114440918</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -555,31 +547,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,J || I |
-|  b,c,d,e,f,g,h,i  || ∅ |</t>
+          <t>| B || A,C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o ||  b,c,d,e,f,g,h,i,j,k,l,m,n  |</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0,0021489859</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0,016231775283813477</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>0,8691401481628418</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -587,31 +578,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>|  A,B,C,D,E,G,H,I  || F |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| L || A,B,C,D,E,F,G,H,I,J,K,M,N,O |
+| ∅ ||       a,c,e,g,i,k,m,o       |</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0,0016031265</t>
+          <t>0,0041897893</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,023689746856689453</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>0,27370142936706543</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -619,31 +609,30 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>|  A,B,C,E,F,G,H,I  || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| G || A,B,C,D,E,F,H,I,J,K,L,M,N,O |
+| ∅ ||        b,d,f,h,j,l,n        |</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,022983789443969727</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>0,22330307960510254</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -651,31 +640,30 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>|  B,C,D,E,G,H,I,J  || F |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| O || A,B,C,D,E,F,G,H,I,J,K,L,M,N |
+| ∅ ||     a,b,d,e,g,h,j,k,m,n     |</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0,0016031265</t>
+          <t>4,7147274e-05</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,023380279541015625</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>0,3995819091796875</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -683,31 +671,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>|  B,C,E,F,G,H,I,J  || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| H || A,B,C,D,E,F,G,I,J,K,L,M,N,O |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>0,022974729537963867</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>1,437063455581665</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -715,31 +702,30 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>|    B,C,D,E,F,H,I    || G |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| H || A,B,C,D,E,F,G,I,J,K,L,M,N,O |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>0,00026786327</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>0,04182577133178711</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>1,477254867553711</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -747,31 +733,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I,J || A |
-|   a,b,d,e,g,h,j   || ∅ |</t>
+          <t>| B || A,C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o ||  b,c,d,e,f,g,h,i,j,k,l,m,n  |</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>0,0013819933</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>0,010632991790771484</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>0,8804044723510742</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -779,31 +764,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H || I |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| B || A,C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o ||  b,c,d,e,f,g,h,i,j,k,l,m,n  |</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0,0021489859</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0,014158487319946289</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>0,8458170890808105</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -811,31 +795,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,J || I |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| L || A,B,C,D,E,F,G,H,I,J,K,M,N,O |
+| ∅ ||       a,c,e,g,i,k,m,o       |</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0,0021489859</t>
+          <t>0,0041897893</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0,01453852653503418</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
+          <t>0,28607845306396484</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -843,31 +826,30 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>|   B,C,D,E,G,H,I   || F |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| G || A,B,C,D,E,F,H,I,J,K,L,M,N,O |
+| ∅ ||        b,d,f,h,j,l,n        |</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>0,0016031265</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0,022724151611328125</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>0,22885870933532715</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -875,31 +857,30 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>|   B,C,E,F,G,H,I   || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| O || A,B,C,D,E,F,G,H,I,J,K,L,M,N |
+| ∅ ||     a,b,d,e,g,h,j,k,m,n     |</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>4,7147274e-05</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0,02129077911376953</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>0,39083194732666016</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -907,31 +888,30 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>|     A,B,D,E,H,J     || G |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| H ||  B,C,D,E,F,G,I,J,K,L,M,N,O  |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0,00026786327</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>0,03912019729614258</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr"/>
+          <t>1,314012050628662</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -939,31 +919,30 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,I || A |
-|  a,b,d,e,g,h,j  || ∅ |</t>
+          <t>| H ||  B,C,D,E,F,G,I,J,K,L,M,N,O  |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0,0013819933</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0,009200572967529297</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr"/>
+          <t>1,2543458938598633</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -971,31 +950,30 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>| B,C,E,F,G,H,I,J || D |
-|  a,b,d,e,g,h,j  || ∅ |</t>
+          <t>| B || C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0,0015337467</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>0,009492158889770508</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr"/>
+          <t>0,789689302444458</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1003,31 +981,30 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>|  B,C,D,E,F,G,H  || I |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| B || C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0,0021489859</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0,013463735580444336</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>0,7249934673309326</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1035,31 +1012,30 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>|    A,B,D,E,G,H    || J |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| L || B,C,D,E,F,G,H,I,J,K,M,N,O |
+| ∅ ||      a,c,e,g,i,k,m,o      |</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0,0017379522</t>
+          <t>0,0041897893</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0,02047276496887207</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>0,23689675331115723</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1067,31 +1043,30 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>|    A,B,E,G,H,J    || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| G || B,C,D,E,F,H,I,J,K,L,M,N,O |
+| ∅ ||       b,d,f,h,j,l,n       |</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0,019946813583374023</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr"/>
+          <t>0,2149944305419922</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1099,31 +1074,30 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>011111100100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>|    B,C,E,F,G,J    || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| O || B,C,D,E,F,G,H,I,J,K,L,M,N |
+| ∅ ||    a,b,d,e,g,h,j,k,m,n    |</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>4,7147274e-05</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0,02002096176147461</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr"/>
+          <t>0,38142848014831543</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1131,31 +1105,30 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H,J || I |
-|     a,c,e,g,i     || ∅ |</t>
+          <t>| H ||  B,C,D,E,F,G,I,J,K,L,M,N,O  |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0,00075376034</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0,007138729095458984</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+          <t>1,2890715599060059</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1163,31 +1136,30 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>| A,B,D,E,F,G,H,I,J || C |
-|     b,d,f,h,j     || ∅ |</t>
+          <t>| H ||  B,C,D,E,F,G,I,J,K,L,M,N,O  |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0,00035369396</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>0,006966352462768555</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr"/>
+          <t>1,2752883434295654</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1195,31 +1167,30 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>| B,C,E,F,G,H,I || D |
-| a,b,d,e,g,h,j || ∅ |</t>
+          <t>| B || C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0,0015337467</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0,008558034896850586</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr"/>
+          <t>0,7357015609741211</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1227,31 +1198,30 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>|       A,C,E,I       || G |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| B || C,D,E,F,G,H,I,J,K,L,M,N,O |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0,00026786327</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0,03431868553161621</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr"/>
+          <t>0,7707915306091309</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1259,31 +1229,30 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>111111111100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>|       B,D,F,H       || J |
-| a,b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| L || B,C,D,E,F,G,H,I,J,K,M,N,O |
+| ∅ ||      a,c,e,g,i,k,m,o      |</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>0,0007697344</t>
+          <t>0,0041897893</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0,036223411560058594</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>0,23595690727233887</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1291,31 +1260,30 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>|   A,B,D,E,G,H   || J |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| G || B,C,D,E,F,H,I,J,K,L,M,N,O |
+| ∅ ||       b,d,f,h,j,l,n       |</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>0,0030118823</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0,012186050415039062</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr"/>
+          <t>0,19769883155822754</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1323,31 +1291,30 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>| A,B,C,D,E,F,G,H || I |
-|    a,c,e,g,i    || ∅ |</t>
+          <t>| O || B,C,D,E,F,G,H,I,J,K,L,M,N |
+| ∅ ||    a,b,d,e,g,h,j,k,m,n    |</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>0,00075376034</t>
+          <t>4,7147274e-05</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0,006409406661987305</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>0,35468411445617676</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1355,31 +1322,30 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>| A,B,D,E,F,G,H,I || C |
-|    b,d,f,h,j    || ∅ |</t>
+          <t>| C ||        A,E,G,I,K,M,O        |
+| n || a,b,c,d,e,f,g,h,i,j,k,l,m,o |</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>0,00035369396</t>
+          <t>0,025339186</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>0,006186962127685547</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>0,48088908195495605</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1387,31 +1353,30 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H,J || I |
-|    a,c,e,g,i    || ∅ |</t>
+          <t>| C ||        A,E,G,I,K,M,O        |
+| n || a,b,c,d,e,f,g,h,i,j,k,l,m,o |</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0,00075376034</t>
+          <t>0,025339186</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>0,006303310394287109</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>0,4814870357513428</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1419,31 +1384,30 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>| B,D,E,F,G,H,I,J || C |
-|    b,d,f,h,j    || ∅ |</t>
+          <t>| C ||       A,E,G,I,K,M,O       |
+| n || b,c,d,e,f,g,h,i,j,k,l,m,o |</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0,00035369396</t>
+          <t>0,025339186</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>0,0065937042236328125</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr"/>
+          <t>0,275068998336792</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1451,31 +1415,30 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>|      A,C,E,G      || I |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| C ||       A,E,G,I,K,M,O       |
+| n || b,c,d,e,f,g,h,i,j,k,l,m,o |</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>0,0031766295</t>
+          <t>0,025339186</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0,017362117767333984</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr"/>
+          <t>0,274127721786499</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1483,31 +1446,30 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>|      A,C,G,I      || E |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| E ||  A,C,G,I,K,M,O  |
+| ∅ || a,c,e,g,i,k,m,o |</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>0,0010385513</t>
+          <t>0,0043781996</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0,01799798011779785</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr"/>
+          <t>0,1088402271270752</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1515,31 +1477,30 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>111111111000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>|      B,D,H,J      || F |
-| a,b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| G || A,C,E,I,K,M,O |
+| ∅ || b,d,f,h,j,l,n |</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>0,0016031265</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0,017155170440673828</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr"/>
+          <t>0,08100318908691406</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1547,31 +1508,30 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>011111111100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>|      B,F,H,J      || D |
-| b,c,d,e,f,g,h,i,j || ∅ |</t>
+          <t>| O ||    A,C,E,G,I,K,M    |
+| ∅ || a,b,d,e,g,h,j,k,m,n |</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>0,0002501011</t>
+          <t>4,7147274e-05</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0,01663517951965332</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>0,13588237762451172</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1579,31 +1539,30 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>|  B,D,E,G,H,J  || A |
-| a,b,d,e,g,h,j || ∅ |</t>
+          <t>| H ||         B,D,F,J,L,N         |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>0,0013819933</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>0,007765531539916992</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr"/>
+          <t>0,36206746101379395</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1611,31 +1570,30 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>| B,C,D,E,F,G,H || I |
-|   a,c,e,g,i   || ∅ |</t>
+          <t>| H ||         B,D,F,J,L,N         |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>0,00075376034</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>0,0052607059478759766</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>0,394317626953125</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1643,31 +1601,30 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>| B,D,E,F,G,H,I || C |
-|   b,d,f,h,j   || ∅ |</t>
+          <t>| B ||        D,F,H,J,L,N        |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>0,00035369396</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>0,0050470829010009766</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>0,22494029998779297</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1675,31 +1632,30 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>|     A,C,E,G     || I |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| B ||        D,F,H,J,L,N        |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>0,0021489859</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>0,009549856185913086</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>0,22421574592590332</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1707,31 +1663,30 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>011111111000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>|     B,D,F,H     || J |
-| b,c,d,e,f,g,h,i || ∅ |</t>
+          <t>| L ||   B,D,F,H,J,N   |
+| ∅ || a,c,e,g,i,k,m,o |</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>0,0030118823</t>
+          <t>0,0041897893</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0,00992131233215332</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr"/>
+          <t>0,07885885238647461</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1739,31 +1694,30 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>|    C,E,G,I    || A |
-| a,b,d,e,g,h,j || ∅ |</t>
+          <t>| N ||  B,D,F,H,J,L  |
+| ∅ || b,d,f,h,j,l,n |</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>0,0013819933</t>
+          <t>0,008794069</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0,00574040412902832</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr"/>
+          <t>0,06245827674865723</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1771,31 +1725,30 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>|    B,F,H,J    || D |
-| a,b,d,e,g,h,j || ∅ |</t>
+          <t>| N ||     B,D,F,H,J,L     |
+| ∅ || a,b,d,e,g,h,j,k,m,n |</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>0,0015337467</t>
+          <t>0,0013378263</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0,005608797073364258</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr"/>
+          <t>0,10491800308227539</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1803,31 +1756,30 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>| A,B,D,E,G,H || J |
-|  a,c,e,g,i  || ∅ |</t>
+          <t>| H ||      A,B,D,E,G,J,K,M,N      |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>0,001448214</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>0,0042302608489990234</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr"/>
+          <t>0,6711196899414062</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1835,31 +1787,30 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>110110110100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>111111111111111</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>| A,B,D,G,H,J || E |
-|  b,d,f,h,j  || ∅ |</t>
+          <t>| H ||      A,B,D,E,G,J,K,M,N      |
+| a || b,c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>0,0019196868</t>
+          <t>0,022765398</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>0,0045282840728759766</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr"/>
+          <t>0,7592926025390625</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1867,31 +1818,30 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>|  A,C,E,G  || I |
-| a,c,e,g,i || ∅ |</t>
+          <t>| B ||     A,D,E,G,H,J,K,M,N     |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>0,00075376034</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>0,0028676986694335938</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr"/>
+          <t>0,40146398544311523</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1899,31 +1849,30 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>011111111111111</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>|  A,E,G,I  || C |
-| b,d,f,h,j || ∅ |</t>
+          <t>| B ||     A,D,E,G,H,J,K,M,N     |
+| o || b,c,d,e,f,g,h,i,j,k,l,m,n |</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0,00035369396</t>
+          <t>0,02527994</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>0,002765178680419922</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr"/>
+          <t>0,4078807830810547</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1931,31 +1880,30 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>101010101000000</t>
+          <t>101010101010101</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>|  B,D,F,H  || J |
-| a,c,e,g,i || ∅ |</t>
+          <t>| E || A,B,D,G,H,J,K,M,N |
+| ∅ ||  a,c,e,g,i,k,m,o  |</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0,001448214</t>
+          <t>0,0043781996</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0,0031032562255859375</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr"/>
+          <t>0,13162660598754883</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1963,31 +1911,92 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>110110110110110</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>010101010100000</t>
+          <t>010101010101010</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>|  D,F,H,J  || B |
-| b,d,f,h,j || ∅ |</t>
+          <t>| G || A,B,D,E,H,J,K,M,N |
+| ∅ ||   b,d,f,h,j,l,n   |</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>0,0034030676</t>
+          <t>0,0070973635</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>0,003070354461669922</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
+          <t>0,7985453605651855</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>110110110110110</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>110110110110110</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>| N ||  A,B,D,E,G,H,J,K,M  |
+| ∅ || a,b,d,e,g,h,j,k,m,n |</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0,0013378263</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0,20035982131958008</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>101111111111111</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>101111111111111</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>| H || A,C,D,E,F,G,I,J,K,L,M,N,O |
+| a || c,d,e,f,g,h,i,j,k,l,m,n,o |</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0,022765398</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0,7356812953948975</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>